<commit_message>
fix: wrap formulas in IFERROR, add age validation, remove dead param, fix identity transform
- Wrap all INDEX/MATCH formulas in IFERROR(...,"") to show empty string
  instead of #N/A for invalid/blank age inputs
- Add whole-number data validation for cell B5 (min=0, max=85)
- Extend data_validations format to support type=whole with formula2
- Remove unused start_row parameter from build_data_table()
- Simplify gender_key derivation by removing redundant .replace() calls

Co-authored-by: petrusjakub <76829088+petrusjakub@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Tabel_Premi_MiUHC.xlsx
+++ b/Tabel_Premi_MiUHC.xlsx
@@ -738,35 +738,35 @@
     </row>
     <row r="9">
       <c r="B9" s="5">
-        <f>INDEX(B$21:B$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(B$21:B$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C9" s="5">
-        <f>INDEX(C$21:C$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(C$21:C$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D9" s="5">
-        <f>INDEX(D$21:D$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(D$21:D$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E9" s="5">
-        <f>INDEX(E$21:E$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(E$21:E$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F9" s="5">
-        <f>INDEX(F$21:F$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(F$21:F$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
       <c r="G9" s="5">
-        <f>INDEX(G$21:G$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(G$21:G$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
       <c r="H9" s="5">
-        <f>INDEX(H$21:H$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(H$21:H$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
       <c r="I9" s="5">
-        <f>INDEX(I$21:I$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0))</f>
+        <f>IFERROR(INDEX(I$21:I$192,MATCH($B$4&amp;"_"&amp;$B$5,$A$21:$A$192,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -795,31 +795,31 @@
     </row>
     <row r="11">
       <c r="B11" s="5">
-        <f>INDEX(B$195:B$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0))</f>
+        <f>IFERROR(INDEX(B$195:B$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C11" s="5">
-        <f>INDEX(C$195:C$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0))</f>
+        <f>IFERROR(INDEX(C$195:C$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D11" s="5">
-        <f>INDEX(D$195:D$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0))</f>
+        <f>IFERROR(INDEX(D$195:D$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E11" s="5">
-        <f>INDEX(E$195:E$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0))</f>
+        <f>IFERROR(INDEX(E$195:E$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F11" s="5">
-        <f>INDEX(F$195:F$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0))</f>
+        <f>IFERROR(INDEX(F$195:F$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0)),"")</f>
         <v>0</v>
       </c>
       <c r="G11" s="5">
-        <f>INDEX(G$195:G$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0))</f>
+        <f>IFERROR(INDEX(G$195:G$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0)),"")</f>
         <v>0</v>
       </c>
       <c r="H11" s="5">
-        <f>INDEX(H$195:H$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0))</f>
+        <f>IFERROR(INDEX(H$195:H$366,MATCH($B$4&amp;"_"&amp;$B$5,$A$195:$A$366,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -857,35 +857,35 @@
     </row>
     <row r="15">
       <c r="B15" s="5">
-        <f>INDEX(B$369:B$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(B$369:B$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C15" s="5">
-        <f>INDEX(C$369:C$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(C$369:C$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D15" s="5">
-        <f>INDEX(D$369:D$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(D$369:D$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E15" s="5">
-        <f>INDEX(E$369:E$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(E$369:E$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F15" s="5">
-        <f>INDEX(F$369:F$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(F$369:F$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
       <c r="G15" s="5">
-        <f>INDEX(G$369:G$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(G$369:G$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
       <c r="H15" s="5">
-        <f>INDEX(H$369:H$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(H$369:H$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
       <c r="I15" s="5">
-        <f>INDEX(I$369:I$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0))</f>
+        <f>IFERROR(INDEX(I$369:I$540,MATCH($B$4&amp;"_"&amp;$B$5,$A$369:$A$540,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -914,31 +914,31 @@
     </row>
     <row r="17">
       <c r="B17" s="5">
-        <f>INDEX(B$543:B$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0))</f>
+        <f>IFERROR(INDEX(B$543:B$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C17" s="5">
-        <f>INDEX(C$543:C$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0))</f>
+        <f>IFERROR(INDEX(C$543:C$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D17" s="5">
-        <f>INDEX(D$543:D$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0))</f>
+        <f>IFERROR(INDEX(D$543:D$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E17" s="5">
-        <f>INDEX(E$543:E$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0))</f>
+        <f>IFERROR(INDEX(E$543:E$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F17" s="5">
-        <f>INDEX(F$543:F$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0))</f>
+        <f>IFERROR(INDEX(F$543:F$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0)),"")</f>
         <v>0</v>
       </c>
       <c r="G17" s="5">
-        <f>INDEX(G$543:G$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0))</f>
+        <f>IFERROR(INDEX(G$543:G$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0)),"")</f>
         <v>0</v>
       </c>
       <c r="H17" s="5">
-        <f>INDEX(H$543:H$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0))</f>
+        <f>IFERROR(INDEX(H$543:H$714,MATCH($B$4&amp;"_"&amp;$B$5,$A$543:$A$714,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -19981,9 +19981,13 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="B4">
       <formula1>"Pria,Wanita"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" sqref="B5">
+      <formula1>0</formula1>
+      <formula2>85</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -20060,35 +20064,35 @@
     </row>
     <row r="9">
       <c r="B9" s="5">
-        <f>INDEX(B$27:B$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(B$27:B$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C9" s="5">
-        <f>INDEX(C$27:C$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(C$27:C$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D9" s="5">
-        <f>INDEX(D$27:D$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(D$27:D$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E9" s="5">
-        <f>INDEX(E$27:E$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(E$27:E$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F9" s="5">
-        <f>INDEX(F$27:F$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(F$27:F$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
       <c r="G9" s="5">
-        <f>INDEX(G$27:G$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(G$27:G$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
       <c r="H9" s="5">
-        <f>INDEX(H$27:H$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(H$27:H$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
       <c r="I9" s="5">
-        <f>INDEX(I$27:I$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0))</f>
+        <f>IFERROR(INDEX(I$27:I$198,MATCH($B$4&amp;"_"&amp;$B$5,$A$27:$A$198,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -20111,23 +20115,23 @@
     </row>
     <row r="11">
       <c r="B11" s="5">
-        <f>INDEX(B$201:B$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0))</f>
+        <f>IFERROR(INDEX(B$201:B$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C11" s="5">
-        <f>INDEX(C$201:C$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0))</f>
+        <f>IFERROR(INDEX(C$201:C$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D11" s="5">
-        <f>INDEX(D$201:D$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0))</f>
+        <f>IFERROR(INDEX(D$201:D$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E11" s="5">
-        <f>INDEX(E$201:E$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0))</f>
+        <f>IFERROR(INDEX(E$201:E$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F11" s="5">
-        <f>INDEX(F$201:F$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0))</f>
+        <f>IFERROR(INDEX(F$201:F$372,MATCH($B$4&amp;"_"&amp;$B$5,$A$201:$A$372,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -20165,35 +20169,35 @@
     </row>
     <row r="15">
       <c r="B15" s="5">
-        <f>INDEX(B$375:B$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(B$375:B$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C15" s="5">
-        <f>INDEX(C$375:C$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(C$375:C$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D15" s="5">
-        <f>INDEX(D$375:D$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(D$375:D$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E15" s="5">
-        <f>INDEX(E$375:E$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(E$375:E$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F15" s="5">
-        <f>INDEX(F$375:F$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(F$375:F$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
       <c r="G15" s="5">
-        <f>INDEX(G$375:G$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(G$375:G$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
       <c r="H15" s="5">
-        <f>INDEX(H$375:H$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(H$375:H$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
       <c r="I15" s="5">
-        <f>INDEX(I$375:I$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0))</f>
+        <f>IFERROR(INDEX(I$375:I$546,MATCH($B$4&amp;"_"&amp;$B$5,$A$375:$A$546,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -20216,23 +20220,23 @@
     </row>
     <row r="17">
       <c r="B17" s="5">
-        <f>INDEX(B$549:B$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0))</f>
+        <f>IFERROR(INDEX(B$549:B$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C17" s="5">
-        <f>INDEX(C$549:C$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0))</f>
+        <f>IFERROR(INDEX(C$549:C$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D17" s="5">
-        <f>INDEX(D$549:D$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0))</f>
+        <f>IFERROR(INDEX(D$549:D$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E17" s="5">
-        <f>INDEX(E$549:E$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0))</f>
+        <f>IFERROR(INDEX(E$549:E$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F17" s="5">
-        <f>INDEX(F$549:F$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0))</f>
+        <f>IFERROR(INDEX(F$549:F$720,MATCH($B$4&amp;"_"&amp;$B$5,$A$549:$A$720,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -20270,35 +20274,35 @@
     </row>
     <row r="21">
       <c r="B21" s="5">
-        <f>INDEX(B$723:B$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(B$723:B$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C21" s="5">
-        <f>INDEX(C$723:C$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(C$723:C$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D21" s="5">
-        <f>INDEX(D$723:D$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(D$723:D$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E21" s="5">
-        <f>INDEX(E$723:E$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(E$723:E$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F21" s="5">
-        <f>INDEX(F$723:F$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(F$723:F$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
       <c r="G21" s="5">
-        <f>INDEX(G$723:G$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(G$723:G$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
       <c r="H21" s="5">
-        <f>INDEX(H$723:H$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(H$723:H$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
       <c r="I21" s="5">
-        <f>INDEX(I$723:I$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0))</f>
+        <f>IFERROR(INDEX(I$723:I$894,MATCH($B$4&amp;"_"&amp;$B$5,$A$723:$A$894,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -20321,23 +20325,23 @@
     </row>
     <row r="23">
       <c r="B23" s="5">
-        <f>INDEX(B$897:B$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0))</f>
+        <f>IFERROR(INDEX(B$897:B$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0)),"")</f>
         <v>0</v>
       </c>
       <c r="C23" s="5">
-        <f>INDEX(C$897:C$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0))</f>
+        <f>IFERROR(INDEX(C$897:C$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0)),"")</f>
         <v>0</v>
       </c>
       <c r="D23" s="5">
-        <f>INDEX(D$897:D$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0))</f>
+        <f>IFERROR(INDEX(D$897:D$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0)),"")</f>
         <v>0</v>
       </c>
       <c r="E23" s="5">
-        <f>INDEX(E$897:E$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0))</f>
+        <f>IFERROR(INDEX(E$897:E$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0)),"")</f>
         <v>0</v>
       </c>
       <c r="F23" s="5">
-        <f>INDEX(F$897:F$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0))</f>
+        <f>IFERROR(INDEX(F$897:F$1068,MATCH($B$4&amp;"_"&amp;$B$5,$A$897:$A$1068,0)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -45783,9 +45787,13 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="B4">
       <formula1>"Pria,Wanita"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" sqref="B5">
+      <formula1>0</formula1>
+      <formula2>85</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>